<commit_message>
JudyP Apparel: rebuild deck + xlsx with cleaned content plan
Picks up the title rewrites and off-brand keyword swaps from
the EmberTribe content-plan.json update.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/judyp-apparel/keyword-research.xlsx
+++ b/decks/judyp-apparel/keyword-research.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Business Casual Women: The Complete Guide</t>
+          <t>Business Casual Women: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Going Out Tops</t>
+          <t>Going Out Tops: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cute Tops</t>
+          <t>Cute Tops: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tunic Clothing</t>
+          <t>Tunic Clothing: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>How to Build a Capsule Wardrobe with Versatile Tops</t>
+          <t>Capsule Wardrobe Tops: Styling Notes and Wardrobe Pairings</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Matching Sets</t>
+          <t>Matching Sets: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Two Piece Sets: The Complete Guide</t>
+          <t>Two Piece Sets: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Dress Shirts</t>
+          <t>Dress Shirts: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Summer Tops</t>
+          <t>Summer Tops: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Blouses: What to Look For</t>
+          <t>Blouses for Women: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Petite Clothing: Sizing Guide</t>
+          <t>Petite Clothing: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Linen Shirt</t>
+          <t>Linen Shirt: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1206,19 +1206,19 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Shirts for Men</t>
+          <t>Lounge Set: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>shirts for men</t>
+          <t>lounge set</t>
         </is>
       </c>
       <c r="D14" s="5" t="n">
-        <v>18100</v>
+        <v>9900</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Button Down Apparel</t>
+          <t>Button Down Apparel: Styling Notes and Wardrobe Pairings</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Clothes for Petite Size: The Complete Guide</t>
+          <t>Clothes for Petite Size: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1347,19 +1347,19 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Women Bag Travel</t>
+          <t>Womens Travel Clothing: The Packable Wardrobe Staple Explained</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>women bag travel</t>
+          <t>womens travel clothing</t>
         </is>
       </c>
       <c r="D17" s="5" t="n">
-        <v>6600</v>
+        <v>1900</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Pillar anchor — highest volume in Wrinkle-Resistant &amp; Travel. Travel use case — JudyP's core customer mindset</t>
+          <t>Travel use case — JudyP's core customer mindset</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Travel Clothes: What to Look For</t>
+          <t>Travel Clothes for Women: What to Pack and How to Wear Them</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Travel use case — JudyP's core customer mindset</t>
+          <t>Pillar anchor — highest volume in Wrinkle-Resistant &amp; Travel. Travel use case — JudyP's core customer mindset</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Travel Outfits: What to Look For</t>
+          <t>Travel Outfits for Women: What to Pack and How to Wear Them</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Best Travelling Clothes for Ladies for 2026</t>
+          <t>The Best Travelling Clothes for Ladies for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Travel Clothes</t>
+          <t>Travel Clothes: Why They're the Smartest Suitcase Choice</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Travel Outfits</t>
+          <t>Travel Outfits: Why They're the Smartest Suitcase Choice</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Travel Dresses</t>
+          <t>Travel Dresses: The Packable Wardrobe Staple Explained</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Travel Sets: What to Look For</t>
+          <t>Travel Sets for Women: A Travel-Friendly Guide for Every Season</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Travel Essentials: What to Look For</t>
+          <t>Travel Essentials for Women: A Travel-Friendly Guide for Every Season</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Rash Guard Women</t>
+          <t>Rash Guard Women: UPF Decoded, Pieces Picked</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>UPF Clothing</t>
+          <t>UPF Clothing: UPF Decoded, Pieces Picked</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Sun Hoodie</t>
+          <t>Sun Hoodie: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Swim Shirt</t>
+          <t>Swim Shirt: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Sun Shirts</t>
+          <t>Sun Shirts: UPF Decoded, Pieces Picked</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Swim Shirts: What to Look For</t>
+          <t>Swim Shirts for Women: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Sunscreen Apparel</t>
+          <t>Sunscreen Apparel: UPF Decoded, Pieces Picked</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>UV Protection Clothing</t>
+          <t>UV Protection Clothing: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Rashguard Women</t>
+          <t>Rashguard Women: UPF Decoded, Pieces Picked</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>American Made Clothing: The Complete Guide</t>
+          <t>American Made Clothing: How to Shop American Without the Guesswork</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Made in USA Clothing: The Complete Guide</t>
+          <t>Made in USA Clothing: How to Shop American Without the Guesswork</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2394,19 +2394,19 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>American Made Shoes: The Complete Guide</t>
+          <t>American Made Clothing for Women: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>american made shoes</t>
+          <t>american made clothing for women</t>
         </is>
       </c>
       <c r="D38" s="5" t="n">
-        <v>3600</v>
+        <v>880</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
@@ -2445,19 +2445,19 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Shoes Made in USA: The Complete Guide</t>
+          <t>American-Made Womens Apparel Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>shoes made in usa</t>
+          <t>american made womens apparel brands</t>
         </is>
       </c>
       <c r="D39" s="5" t="n">
-        <v>3600</v>
+        <v>590</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Compare</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -2496,23 +2496,23 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>American Jeans</t>
+          <t>Clothing Made in the United States: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>american jeans</t>
+          <t>clothing made in the united states</t>
         </is>
       </c>
       <c r="D40" s="5" t="n">
-        <v>2900</v>
+        <v>1300</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>32</v>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G40" s="13" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Clothing Makers in USA: The Complete Guide</t>
+          <t>Clothing Makers in USA: How to Shop American Without the Guesswork</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Apparel Petite: Sizing Guide</t>
+          <t>Apparel Petite: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Best Clothing Linen Shirt for 2026</t>
+          <t>The Best Clothing Linen Shirt for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Oxford Shirt: The Complete Guide</t>
+          <t>Oxford Shirt: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Matching Sets Women</t>
+          <t>Matching Sets Women: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>2 Piece Sets</t>
+          <t>2 Piece Sets: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Best Athletic Dress for 2026</t>
+          <t>The Best Athletic Dress for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Vacation Outfits</t>
+          <t>Vacation Outfits: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -2923,23 +2923,23 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Top Women Tops</t>
+          <t>The Best White Button Up Blouse Womens for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>top women tops</t>
+          <t>white button up blouse womens</t>
         </is>
       </c>
       <c r="D49" s="5" t="n">
-        <v>12100</v>
+        <v>8100</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="F49" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>38</v>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Decision</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Women Tops</t>
+          <t>Women Tops: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Cute Shirts</t>
+          <t>Cute Shirts: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Two Piece Sets Women</t>
+          <t>Two Piece Sets Women: Styling Notes and Wardrobe Pairings</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Women Clothes</t>
+          <t>Women Clothes: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Garments Brands Worth Knowing</t>
+          <t>Garments Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Ladies Interview Clothes</t>
+          <t>Ladies Interview Clothes: Styling Notes and Wardrobe Pairings</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Trendy Wear for Ladies: The Complete Guide</t>
+          <t>Trendy Wear for Ladies: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Travel Set</t>
+          <t>Travel Set: A Travel-Friendly Guide for Every Season</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Travel Accessories: What to Look For</t>
+          <t>Travel Accessories for Women: The Packable Wardrobe Staple Explained</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Travel Necessities: The Complete Guide</t>
+          <t>Travel Necessities: What to Pack and How to Wear Them</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Wrinkle Free Dress Shirts</t>
+          <t>Wrinkle Free Dress Shirts: Why They're the Smartest Suitcase Choice</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Wrinkle Free Shirts</t>
+          <t>Wrinkle Free Shirts: The Packable Wardrobe Staple Explained</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Travel Gear</t>
+          <t>Travel Gear: What to Pack and How to Wear Them</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Wrinkle Free Travel Clothes</t>
+          <t>Wrinkle Free Travel Clothes: A Travel-Friendly Guide for Every Season</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Sun Shirts: What to Look For</t>
+          <t>Sun Shirts for Women: What UPF Actually Means and Which Pieces Earn It</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3864,23 +3864,23 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Swimming Shirts for Guys</t>
+          <t>Sun Protection Clothing: How to Stay Covered Without Sacrificing Style</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>swimming shirts for guys</t>
+          <t>sun protection clothing</t>
         </is>
       </c>
       <c r="D68" s="5" t="n">
-        <v>2900</v>
+        <v>5400</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="F68" s="8" t="inlineStr">
-        <is>
-          <t>Easy</t>
+        <v>47</v>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="G68" s="11" t="inlineStr">
@@ -3895,7 +3895,7 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
@@ -3911,19 +3911,19 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>Sun Shirts for Men</t>
+          <t>SPF Shirts: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>sun shirts for men</t>
+          <t>spf shirts</t>
         </is>
       </c>
       <c r="D69" s="5" t="n">
         <v>2400</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F69" s="8" t="inlineStr">
         <is>
@@ -3942,7 +3942,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>Compare</t>
+          <t>Info</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3950,7 +3950,11 @@
           <t>M2</t>
         </is>
       </c>
-      <c r="K69" s="3" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Sun-protective product category — high commercial intent</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3958,7 +3962,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Best Long Sleeve Swimsuit Women for 2026</t>
+          <t>The Best Long Sleeve Swimsuit Women for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -4009,7 +4013,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Wear Sun Protection: The Complete Guide</t>
+          <t>Wear Sun Protection: What UPF Actually Means and Which Pieces Earn It</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -4056,7 +4060,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Best Female Swimming Suits for 2026</t>
+          <t>The Best Female Swimming Suits for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -4103,7 +4107,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>UPF Vs SPF: The Complete Guide</t>
+          <t>UPF Vs SPF: How to Stay Covered Without Sacrificing Style</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -4154,7 +4158,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Ultraviolet Protection Clothing: The Complete Guide</t>
+          <t>Ultraviolet Protection Clothing: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -4201,7 +4205,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Clothing Mfg USA: The Complete Guide</t>
+          <t>Clothing Mfg USA: How to Shop American Without the Guesswork</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4248,7 +4252,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>America Shirt</t>
+          <t>America Shirt: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4295,7 +4299,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Clothing USA Brands Worth Knowing</t>
+          <t>Clothing USA Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4342,7 +4346,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>American Made Clothing Brands Worth Knowing</t>
+          <t>American Made Clothing Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4393,7 +4397,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>American Clothing Brands Made in America Worth Knowing</t>
+          <t>American Clothing Brands Made in America: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4440,19 +4444,19 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>American Style Men</t>
+          <t>Dresses Made in USA: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>american style men</t>
+          <t>dresses made in usa</t>
         </is>
       </c>
       <c r="D80" s="5" t="n">
-        <v>1600</v>
+        <v>880</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
@@ -4481,7 +4485,7 @@
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Easy win — fast indexing expected</t>
+          <t>Easy win — fast indexing expected. Made-in-USA positioning — direct brand alignment</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4495,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Garments Made in USA</t>
+          <t>Garments Made in USA: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4542,7 +4546,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Work on Clothes: The Complete Guide</t>
+          <t>Work on Clothes: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -4589,7 +4593,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Popular Clothing Brands Worth Knowing</t>
+          <t>Popular Clothing Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4636,7 +4640,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Shirt with Button Down: The Complete Guide</t>
+          <t>Shirt with Button Down: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4683,7 +4687,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Business Casual Outfits: The Complete Guide</t>
+          <t>Business Casual Outfits: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -4730,7 +4734,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Made in the States: The Complete Guide</t>
+          <t>Made in the States: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -4777,7 +4781,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Best White Button Down Shirt for 2026</t>
+          <t>The Best White Button Down Shirt for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4828,7 +4832,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Business Casual Attire for Women: The Complete Guide</t>
+          <t>Business Casual Attire for Women: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4875,7 +4879,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Business Attire Women: The Complete Guide</t>
+          <t>Business Attire Women: How to Wear Them Three Ways</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4922,7 +4926,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Best Button Down Shirts for Women for 2026</t>
+          <t>The Best Button Down Shirts for Women for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4969,7 +4973,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Business Casuals for Ladies: The Complete Guide</t>
+          <t>Business Casuals for Ladies: Styling Notes and Wardrobe Pairings</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -5016,7 +5020,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Famous Garment Brands Worth Knowing</t>
+          <t>Famous Garment Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -5063,7 +5067,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Business Professional Attire Women: The Complete Guide</t>
+          <t>Business Professional Attire Women: What Makes One Worth Buying</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -5110,7 +5114,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>Best White Button Up for 2026</t>
+          <t>The Best White Button Up for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -5157,7 +5161,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Known Brands Clothing Worth Knowing</t>
+          <t>Known Brands Clothing: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -5204,7 +5208,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Best Linen Shirt Women for 2026</t>
+          <t>The Best Linen Shirt Women for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5357,7 +5361,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Capsule Wardrobe for Travel: The Complete Guide</t>
+          <t>Capsule Wardrobe for Travel: Why They're the Smartest Suitcase Choice</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -5408,7 +5412,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Quick Drying: The Complete Guide</t>
+          <t>Quick Drying: A Travel-Friendly Guide for Every Season</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -5455,7 +5459,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Airport Travel Outfits: The Complete Guide</t>
+          <t>Airport Travel Outfits: What to Pack and How to Wear Them</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -5506,7 +5510,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Summer Travel Outfits: The Complete Guide</t>
+          <t>Summer Travel Outfits: What to Pack and How to Wear Them</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -5557,7 +5561,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Traveling Essentials: The Complete Guide</t>
+          <t>Traveling Essentials: The Packable Wardrobe Staple Explained</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -5608,7 +5612,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Travel Outfit Ideas</t>
+          <t>Travel Outfit Ideas: Outfit Inspiration for Real Life</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -5659,7 +5663,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Does Lyocell Wrinkle: The Complete Guide</t>
+          <t>Does Lyocell Wrinkle: The Packable Wardrobe Staple Explained</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -5710,7 +5714,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Airport Travel Outfit Ideas</t>
+          <t>Airport Travel Outfit Ideas: Outfit Inspiration for Real Life</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -5761,7 +5765,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Protect from Sunlight: The Complete Guide</t>
+          <t>Protect From Sunlight: UPF Decoded, Pieces Picked</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -5808,7 +5812,7 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Sun Protection Shirts: The Complete Guide</t>
+          <t>Sun Protection Shirts: A Sun-Safe Wardrobe Guide</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -5855,7 +5859,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>UPF 50 Sun Protection Clothing: The Complete Guide</t>
+          <t>UPF 50 Sun Protection Clothing: How to Stay Covered Without Sacrificing Style</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -5906,7 +5910,7 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>UPF Meaning</t>
+          <t>UPF Meaning: Definition, Origins, and How to Wear It</t>
         </is>
       </c>
       <c r="C110" s="4" t="inlineStr">
@@ -5957,7 +5961,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Best Hooded Sun Shirt for 2026</t>
+          <t>The Best Hooded Sun Shirt for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -6008,7 +6012,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>Best Long Sleeve Swim Suit for 2026</t>
+          <t>The Best Long Sleeve Swim Suit for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
@@ -6106,7 +6110,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Best Swim Rash Guard for 2026</t>
+          <t>The Best Swim Rash Guard for 2026 (and How to Choose)</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
@@ -6153,7 +6157,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Clothing Brands Made in USA Worth Knowing</t>
+          <t>Clothing Brands Made in USA: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -6204,7 +6208,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Made in America Clothing</t>
+          <t>Made in America Clothing: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
@@ -6251,7 +6255,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>American Made T Shirts</t>
+          <t>American Made T Shirts: A Field Guide to American-Made Pieces</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -6302,7 +6306,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>American Brands Worth Knowing</t>
+          <t>American Brands: Names Worth Knowing</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -6349,28 +6353,28 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>American Garment Manufacturers</t>
+          <t>Cotton 3/4 Sleeve Tops for Women: A Smart-Casual Essentials Guide</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>american garment manufacturers</t>
+          <t>cotton 3/4 sleeve tops for women</t>
         </is>
       </c>
       <c r="D119" s="5" t="n">
-        <v>1600</v>
+        <v>720</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="F119" s="8" t="inlineStr">
         <is>
           <t>Easy</t>
         </is>
       </c>
-      <c r="G119" s="13" t="inlineStr">
-        <is>
-          <t>Made in USA</t>
+      <c r="G119" s="7" t="inlineStr">
+        <is>
+          <t>Versatile &amp; Smart-Casual</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -6396,23 +6400,23 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Clothing Manufacturers in USA</t>
+          <t>American Shirts: Where They're Made and Why It Matters</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>clothing manufacturers in usa</t>
+          <t>american shirts</t>
         </is>
       </c>
       <c r="D120" s="5" t="n">
-        <v>1600</v>
+        <v>880</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="F120" s="6" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+        <v>21</v>
+      </c>
+      <c r="F120" s="8" t="inlineStr">
+        <is>
+          <t>Easy</t>
         </is>
       </c>
       <c r="G120" s="13" t="inlineStr">
@@ -6443,7 +6447,7 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>USA Shirt</t>
+          <t>USA Shirt: How to Shop American Without the Guesswork</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">
@@ -7377,12 +7381,12 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -7795,12 +7799,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Bottom of funnel</t>
-        </is>
-      </c>
-      <c r="H34" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -8099,12 +8103,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H42" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H42" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9201,12 +9205,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H71" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Bottom of funnel</t>
+        </is>
+      </c>
+      <c r="H71" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -9923,12 +9927,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H90" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H90" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -10721,12 +10725,12 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H111" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H111" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -12244,9 +12248,9 @@
           <t>Top of funnel</t>
         </is>
       </c>
-      <c r="H151" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="H151" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -12282,9 +12286,9 @@
           <t>Top of funnel</t>
         </is>
       </c>
-      <c r="H152" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+      <c r="H152" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -13761,12 +13765,12 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H191" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H191" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -15585,12 +15589,12 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H239" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H239" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -17371,12 +17375,12 @@
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H286" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H286" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -18017,12 +18021,12 @@
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H303" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H303" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -22197,12 +22201,12 @@
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H413" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H413" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -22577,12 +22581,12 @@
       </c>
       <c r="G423" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H423" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H423" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -24743,12 +24747,12 @@
       </c>
       <c r="G480" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H480" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H480" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -24781,12 +24785,12 @@
       </c>
       <c r="G481" t="inlineStr">
         <is>
-          <t>Middle of funnel</t>
-        </is>
-      </c>
-      <c r="H481" s="14" t="inlineStr">
-        <is>
-          <t>Yes (planned)</t>
+          <t>Top of funnel</t>
+        </is>
+      </c>
+      <c r="H481" s="15" t="inlineStr">
+        <is>
+          <t>Overflow</t>
         </is>
       </c>
     </row>
@@ -27099,12 +27103,12 @@
       </c>
       <c r="G542" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H542" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H542" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -35082,9 +35086,9 @@
           <t>Top of funnel</t>
         </is>
       </c>
-      <c r="H752" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+      <c r="H752" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -35117,12 +35121,12 @@
       </c>
       <c r="G753" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H753" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H753" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>
@@ -35193,12 +35197,12 @@
       </c>
       <c r="G755" t="inlineStr">
         <is>
-          <t>Top of funnel</t>
-        </is>
-      </c>
-      <c r="H755" s="15" t="inlineStr">
-        <is>
-          <t>Overflow</t>
+          <t>Middle of funnel</t>
+        </is>
+      </c>
+      <c r="H755" s="14" t="inlineStr">
+        <is>
+          <t>Yes (planned)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
JudyP Apparel: rebuild deck + xlsx with diverse titles
Picks up the wide-angle title rewrite — 119/120 unique titles across
the 120-article plan.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/judyp-apparel/keyword-research.xlsx
+++ b/decks/judyp-apparel/keyword-research.xlsx
@@ -638,7 +638,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Business Casual Women: How to Wear Them Three Ways</t>
+          <t>Business Casual Women: From Boardroom to Brunch</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Going Out Tops: A Smart-Casual Essentials Guide</t>
+          <t>Why Going Out Tops Earn a Permanent Spot in Your Wardrobe</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Cute Tops: How to Wear Them Three Ways</t>
+          <t>What Smart-Casual Actually Means for Cute Tops</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Tunic Clothing: How to Wear Them Three Ways</t>
+          <t>Tunic Clothing: A Guide to Fit, Fabric, and Finish</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Capsule Wardrobe Tops: Styling Notes and Wardrobe Pairings</t>
+          <t>The Honest Verdict on Capsule Wardrobe Tops</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -877,7 +877,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Matching Sets: A Smart-Casual Essentials Guide</t>
+          <t>How a Single Matching Set Can Anchor Five Outfits</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Two Piece Sets: How to Wear Them Three Ways</t>
+          <t>Two Piece Sets: A Plain-English Guide to a Better Closet</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Dress Shirts: A Smart-Casual Essentials Guide</t>
+          <t>Building a Wardrobe Around Dress Shirts</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Summer Tops: How to Wear Them Three Ways</t>
+          <t>How Summer Tops Pair with Everything You Already Own</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Blouses for Women: A Smart-Casual Essentials Guide</t>
+          <t>Blouses for Women: The Real Difference Between $40 and $140</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Petite Clothing: How to Wear Them Three Ways</t>
+          <t>Petite Clothing: The Editor's Notes on What Actually Works</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Linen Shirt: What Makes One Worth Buying</t>
+          <t>Linen Shirt: How to Build the Capsule Around Them</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1206,7 +1206,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Lounge Set: A Smart-Casual Essentials Guide</t>
+          <t>Lounge Set: A Plain-English Guide to a Better Closet</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1253,7 +1253,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Button Down Apparel: Styling Notes and Wardrobe Pairings</t>
+          <t>Button Down Apparel: The Tactile Difference That Sells Itself</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Clothes for Petite Size: How to Wear Them Three Ways</t>
+          <t>Clothes for Petite Size: A Year of Wearing the Same Three Pieces</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Womens Travel Clothing: The Packable Wardrobe Staple Explained</t>
+          <t>Womens Travel Clothing: Why Tencel Beats Polyester for the Long Flight</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Travel Clothes for Women: What to Pack and How to Wear Them</t>
+          <t>The Quiet Magic of Travel Clothes for Women</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1449,7 +1449,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Travel Outfits for Women: What to Pack and How to Wear Them</t>
+          <t>From Plane to Restaurant: Styling Travel Outfits for Women</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>The Best Travelling Clothes for Ladies for 2026 (and How to Choose)</t>
+          <t>Travelling Clothes for Ladies: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Travel Clothes: Why They're the Smartest Suitcase Choice</t>
+          <t>Travel Clothes: The Pieces That Actually Survive a Suitcase</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1602,7 +1602,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Travel Outfits: Why They're the Smartest Suitcase Choice</t>
+          <t>Travel Outfits: The Travel Editor's Take</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Travel Dresses: The Packable Wardrobe Staple Explained</t>
+          <t>From Plane to Restaurant: Styling Travel Dresses</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1704,7 +1704,7 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Travel Sets for Women: A Travel-Friendly Guide for Every Season</t>
+          <t>A Smarter Way to Pack: Starting With Travel Sets for Women</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Best Travel Accessories (2026 Buyer's Guide)</t>
+          <t>Best Travel Accessories Worth Your Money in 2026</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1806,7 +1806,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Travel Essentials for Women: A Travel-Friendly Guide for Every Season</t>
+          <t>Travel Essentials for Women: One Outfit, Three Climates</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Rash Guard Women: UPF Decoded, Pieces Picked</t>
+          <t>The Sun-Smart Wardrobe: Starting With Rash Guard Women</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>UPF Clothing: UPF Decoded, Pieces Picked</t>
+          <t>Reading the Tag: How to Spot Real Sun Protection in UPF Clothing</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Sun Hoodie: A Sun-Safe Wardrobe Guide</t>
+          <t>Sun Hoodie: A Plain-English Guide to UPF Ratings</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Swim Shirt: A Sun-Safe Wardrobe Guide</t>
+          <t>Swim Shirt: A Plain-English Guide to UPF Ratings</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Sun Shirts: UPF Decoded, Pieces Picked</t>
+          <t>The Sun-Smart Wardrobe: Starting With Sun Shirts</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Swim Shirts for Women: A Sun-Safe Wardrobe Guide</t>
+          <t>Swim Shirts for Women for Beach Days, Boat Days, and Garden Days</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Sunscreen Apparel: UPF Decoded, Pieces Picked</t>
+          <t>How Sunscreen Apparel Earn Their UPF Rating (and How to Verify)</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>UV Protection Clothing: A Sun-Safe Wardrobe Guide</t>
+          <t>UV Protection Clothing: Lightweight Coverage for Hot Weather</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Rashguard Women: UPF Decoded, Pieces Picked</t>
+          <t>What Makes a UPF Garment Worth the Label</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2292,7 +2292,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>American Made Clothing: How to Shop American Without the Guesswork</t>
+          <t>American Made Clothing for Shoppers Who Read the Tag First</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Made in USA Clothing: How to Shop American Without the Guesswork</t>
+          <t>Made in USA Clothing: A Buyer's Guide to Garments Still Made on US Soil</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>American Made Clothing for Women: A Field Guide to American-Made Pieces</t>
+          <t>American Made Clothing for Women: The Real Story Behind the Label</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -2445,7 +2445,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>American-Made Womens Apparel Brands: Names Worth Knowing</t>
+          <t>American Made Womens Apparel Brands: The Quality You Can Trace to a Mill</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -2496,7 +2496,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Clothing Made in the United States: A Field Guide to American-Made Pieces</t>
+          <t>From Cut and Sew to Hangtag: How Clothing Made in the United States Get Made</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -2543,7 +2543,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Clothing Makers in USA: How to Shop American Without the Guesswork</t>
+          <t>Clothing Makers in USA: A Year of Wearing American-Made</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Apparel Petite: What Makes One Worth Buying</t>
+          <t>Apparel Petite: When to Spend, When to Skip</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>The Best Clothing Linen Shirt for 2026 (and How to Choose)</t>
+          <t>Clothing Linen Shirt: What to Buy, What to Skip</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Oxford Shirt: What Makes One Worth Buying</t>
+          <t>Oxford Shirt: A Plain-English Guide to a Better Closet</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -2735,7 +2735,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Matching Sets Women: What Makes One Worth Buying</t>
+          <t>Matching Sets Women: From Boardroom to Brunch</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>2 Piece Sets: How to Wear Them Three Ways</t>
+          <t>The Honest Verdict on 2 Piece Sets</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -2829,7 +2829,7 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>The Best Athletic Dress for 2026 (and How to Choose)</t>
+          <t>Athletic Dress: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Vacation Outfits: How to Wear Them Three Ways</t>
+          <t>Why Vacation Outfits Earn a Permanent Spot in Your Wardrobe</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -2923,7 +2923,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>The Best White Button Up Blouse Womens for 2026 (and How to Choose)</t>
+          <t>White Button Up Blouse Womens: A Considered Buyer's Guide</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Women Tops: What Makes One Worth Buying</t>
+          <t>Women Tops: The Real Difference Between $40 and $140</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Cute Shirts: A Smart-Casual Essentials Guide</t>
+          <t>Cute Shirts: A Buying Lens for the Long Run</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Two Piece Sets Women: Styling Notes and Wardrobe Pairings</t>
+          <t>Two Piece Sets Women: A Wardrobe Audit Starting Point</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Women Clothes: What Makes One Worth Buying</t>
+          <t>Building a Wardrobe Around Women Clothes</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Garments Brands: Names Worth Knowing</t>
+          <t>Garments Brands: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Ladies Interview Clothes: Styling Notes and Wardrobe Pairings</t>
+          <t>The Honest Verdict on Ladies Interview Clothes</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Trendy Wear for Ladies: A Smart-Casual Essentials Guide</t>
+          <t>Why Trendy Wear for Ladies Are the Most-Worn Item in a Smart Wardrobe</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Best Travel Clothes for Women (2026 Buyer's Guide)</t>
+          <t>Choosing Best Travel Clothes for Women: A Decision Framework</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Best Travel Bags for Women (2026 Buyer's Guide)</t>
+          <t>Best Travel Bags for Women: The Brands Quietly Doing It Right</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Travel Set: A Travel-Friendly Guide for Every Season</t>
+          <t>The Case for Travel Set on Long-Haul Days</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3456,7 +3456,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Travel Accessories for Women: The Packable Wardrobe Staple Explained</t>
+          <t>Travel Accessories for Women: One Outfit, Three Climates</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Travel Necessities: What to Pack and How to Wear Them</t>
+          <t>Travel Necessities: How to Wear One Top Five Ways</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Wrinkle Free Dress Shirts: Why They're the Smartest Suitcase Choice</t>
+          <t>Wrinkle Free Dress Shirts That Look Pressed After Twelve Hours in Flight</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Wrinkle Free Shirts: The Packable Wardrobe Staple Explained</t>
+          <t>Wrinkle Free Shirts: The Travel Editor's Take</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Travel Gear: What to Pack and How to Wear Them</t>
+          <t>Travel Gear: Why Tencel Beats Polyester for the Long Flight</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Wrinkle Free Travel Clothes: A Travel-Friendly Guide for Every Season</t>
+          <t>How Wrinkle Free Travel Clothes Earn Repeat Trips</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
@@ -3762,7 +3762,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Best Travel Items (2026 Buyer's Guide)</t>
+          <t>Best of 2026: Best Travel Items That Stood Out</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Sun Shirts for Women: What UPF Actually Means and Which Pieces Earn It</t>
+          <t>From Hiking to Brunch: Sun Shirts for Women That Cover All Day</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Sun Protection Clothing: How to Stay Covered Without Sacrificing Style</t>
+          <t>The Sun-Smart Wardrobe: Starting With Sun Protection Clothing</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -3911,7 +3911,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>SPF Shirts: A Sun-Safe Wardrobe Guide</t>
+          <t>SPF Shirts That Don't Look Like Sun Protection</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>The Best Long Sleeve Swimsuit Women for 2026 (and How to Choose)</t>
+          <t>Choosing Long Sleeve Swimsuit Women: A Decision Framework</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -4013,7 +4013,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Wear Sun Protection: What UPF Actually Means and Which Pieces Earn It</t>
+          <t>Wear Sun Protection: Stylish Coverage That Still Breathes</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -4060,7 +4060,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>The Best Female Swimming Suits for 2026 (and How to Choose)</t>
+          <t>Female Swimming Suits: A Considered Buyer's Guide</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>UPF Vs SPF: How to Stay Covered Without Sacrificing Style</t>
+          <t>UPF Vs SPF: A Side-by-Side Comparison</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Ultraviolet Protection Clothing: A Sun-Safe Wardrobe Guide</t>
+          <t>The Sun-Smart Wardrobe: Starting With Ultraviolet Protection Clothing</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Clothing Mfg USA: How to Shop American Without the Guesswork</t>
+          <t>Inside a US Garment Factory: How Clothing Mfg USA Are Built</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>America Shirt: A Field Guide to American-Made Pieces</t>
+          <t>How to Spot Real America Shirt on a Hangtag</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Clothing USA Brands: Names Worth Knowing</t>
+          <t>Clothing USA Brands: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4346,7 +4346,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>American Made Clothing Brands: Names Worth Knowing</t>
+          <t>American Made Clothing Brands: A Considered Buyer's Guide</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>American Clothing Brands Made in America: Names Worth Knowing</t>
+          <t>American Clothing Brands Made in America: The Brands Quietly Doing It Right</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4444,7 +4444,7 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Dresses Made in USA: A Field Guide to American-Made Pieces</t>
+          <t>Dresses Made in USA: A Living List of Brands Worth Supporting</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Garments Made in USA: A Field Guide to American-Made Pieces</t>
+          <t>Garments Made in USA: The Real Story Behind the Label</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Work on Clothes: A Smart-Casual Essentials Guide</t>
+          <t>Work on Clothes: A Wardrobe Audit Starting Point</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -4593,7 +4593,7 @@
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Popular Clothing Brands: Names Worth Knowing</t>
+          <t>The Short List: Popular Clothing Brands Worth Considering</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4640,7 +4640,7 @@
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Shirt with Button Down: A Smart-Casual Essentials Guide</t>
+          <t>Shirt with Button Down: When to Spend, When to Skip</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Business Casual Outfits: How to Wear Them Three Ways</t>
+          <t>Business Casual Outfits: A Year of Wearing the Same Three Pieces</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -4734,7 +4734,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Made in the States: How to Wear Them Three Ways</t>
+          <t>The Honest Verdict on Made in the States</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -4781,7 +4781,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>The Best White Button Down Shirt for 2026 (and How to Choose)</t>
+          <t>White Button Down Shirt: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -4832,7 +4832,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Business Casual Attire for Women: How to Wear Them Three Ways</t>
+          <t>Business Casual Attire for Women: A Plain-English Guide to a Better Closet</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -4879,7 +4879,7 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Business Attire Women: How to Wear Them Three Ways</t>
+          <t>Business Attire Women: A Wardrobe Audit Starting Point</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -4926,7 +4926,7 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>The Best Button Down Shirts for Women for 2026 (and How to Choose)</t>
+          <t>The Best Button Down Shirts for Women for 2026</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Business Casuals for Ladies: Styling Notes and Wardrobe Pairings</t>
+          <t>Business Casuals for Ladies: Three Outfits, One Top, One Week</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Famous Garment Brands: Names Worth Knowing</t>
+          <t>What Makes Famous Garment Brands Worth Replacing Every Few Years</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -5067,7 +5067,7 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Business Professional Attire Women: What Makes One Worth Buying</t>
+          <t>How to Get More Years Out of Business Professional Attire Women</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>The Best White Button Up for 2026 (and How to Choose)</t>
+          <t>What Makes White Button Up Worth Replacing Every Few Years</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Known Brands Clothing: Names Worth Knowing</t>
+          <t>Known Brands Clothing: A Buyer's Guide for Real Shoppers</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>The Best Linen Shirt Women for 2026 (and How to Choose)</t>
+          <t>Linen Shirt Women: What to Buy, What to Skip</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5259,7 +5259,7 @@
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>Best Travel Clothes (2026 Buyer's Guide)</t>
+          <t>Best Travel Clothes: A Buyer's Guide for Real Shoppers</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Best Travel Outfits (2026 Buyer's Guide)</t>
+          <t>Best Travel Outfits: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -5361,7 +5361,7 @@
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Capsule Wardrobe for Travel: Why They're the Smartest Suitcase Choice</t>
+          <t>Capsule Wardrobe for Travel That Look Pressed After Twelve Hours in Flight</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Quick Drying: A Travel-Friendly Guide for Every Season</t>
+          <t>Quick Drying: Fabric Notes from the JudyP Studio</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -5459,7 +5459,7 @@
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Airport Travel Outfits: What to Pack and How to Wear Them</t>
+          <t>How to Pack Airport Travel Outfits So They Stay Crisp</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Summer Travel Outfits: What to Pack and How to Wear Them</t>
+          <t>Summer Travel Outfits: Why Tencel Beats Polyester for the Long Flight</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Traveling Essentials: The Packable Wardrobe Staple Explained</t>
+          <t>The Quiet Magic of Traveling Essentials</t>
         </is>
       </c>
       <c r="C103" s="4" t="inlineStr">
@@ -5612,7 +5612,7 @@
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>Travel Outfit Ideas: Outfit Inspiration for Real Life</t>
+          <t>A Packing List Built Around Travel Outfit Ideas</t>
         </is>
       </c>
       <c r="C104" s="4" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Does Lyocell Wrinkle: The Packable Wardrobe Staple Explained</t>
+          <t>Does Lyocell Wrinkle: What to Pack for a Two-Week Trip</t>
         </is>
       </c>
       <c r="C105" s="4" t="inlineStr">
@@ -5714,7 +5714,7 @@
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Airport Travel Outfit Ideas: Outfit Inspiration for Real Life</t>
+          <t>Why Airport Travel Outfit Ideas Earn Their Spot in a Carry-On</t>
         </is>
       </c>
       <c r="C106" s="4" t="inlineStr">
@@ -5765,7 +5765,7 @@
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Protect From Sunlight: UPF Decoded, Pieces Picked</t>
+          <t>How Protect from Sunlight Compare to Sunscreen (and Why You Want Both)</t>
         </is>
       </c>
       <c r="C107" s="4" t="inlineStr">
@@ -5812,7 +5812,7 @@
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Sun Protection Shirts: A Sun-Safe Wardrobe Guide</t>
+          <t>Sun Protection Shirts That Don't Look Like Sun Protection</t>
         </is>
       </c>
       <c r="C108" s="4" t="inlineStr">
@@ -5859,7 +5859,7 @@
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>UPF 50 Sun Protection Clothing: How to Stay Covered Without Sacrificing Style</t>
+          <t>What Makes a UPF Garment Worth the Label</t>
         </is>
       </c>
       <c r="C109" s="4" t="inlineStr">
@@ -5961,7 +5961,7 @@
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>The Best Hooded Sun Shirt for 2026 (and How to Choose)</t>
+          <t>Hooded Sun Shirt: What to Buy, What to Skip</t>
         </is>
       </c>
       <c r="C111" s="4" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>The Best Long Sleeve Swim Suit for 2026 (and How to Choose)</t>
+          <t>Long Sleeve Swim Suit: A Comparison You Can Actually Use</t>
         </is>
       </c>
       <c r="C112" s="4" t="inlineStr">
@@ -6063,7 +6063,7 @@
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Best Sun Shirts (2026 Buyer's Guide)</t>
+          <t>Best Sun Shirts Worth Your Money in 2026</t>
         </is>
       </c>
       <c r="C113" s="4" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>The Best Swim Rash Guard for 2026 (and How to Choose)</t>
+          <t>How to Pick Swim Rash Guard That Outlast the Trend</t>
         </is>
       </c>
       <c r="C114" s="4" t="inlineStr">
@@ -6157,7 +6157,7 @@
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Clothing Brands Made in USA: Names Worth Knowing</t>
+          <t>What Makes Clothing Brands Made in USA Worth Replacing Every Few Years</t>
         </is>
       </c>
       <c r="C115" s="4" t="inlineStr">
@@ -6208,7 +6208,7 @@
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Made in America Clothing: A Field Guide to American-Made Pieces</t>
+          <t>Made in America Clothing: The Real Story Behind the Label</t>
         </is>
       </c>
       <c r="C116" s="4" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>American Made T Shirts: A Field Guide to American-Made Pieces</t>
+          <t>Where American Made T Shirts Are Actually Made (and How to Check)</t>
         </is>
       </c>
       <c r="C117" s="4" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>American Brands: Names Worth Knowing</t>
+          <t>American Brands: A Year-Long Review of What Actually Lasts</t>
         </is>
       </c>
       <c r="C118" s="4" t="inlineStr">
@@ -6353,7 +6353,7 @@
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Cotton 3/4 Sleeve Tops for Women: A Smart-Casual Essentials Guide</t>
+          <t>Cotton 3/4 Sleeve Tops for Women: A Year of Wearing the Same Three Pieces</t>
         </is>
       </c>
       <c r="C119" s="4" t="inlineStr">
@@ -6400,7 +6400,7 @@
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>American Shirts: Where They're Made and Why It Matters</t>
+          <t>American Shirts: The Brands Still Manufacturing in America</t>
         </is>
       </c>
       <c r="C120" s="4" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>USA Shirt: How to Shop American Without the Guesswork</t>
+          <t>Why USA Shirt Feel Different on the Body</t>
         </is>
       </c>
       <c r="C121" s="4" t="inlineStr">

</xml_diff>